<commit_message>
feat(F-NAR-019): ATOM-AUT.AFF.001-06 La pomme du marché
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-AUT.AFF.001-06.xlsx
+++ b/stories/arbres/ATOM-AUT.AFF.001-06.xlsx
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Nina veut une pomme brillante au hall. Elle pose une cuillère, la retire, trouve le chapeau. La pomme est froide dans sa main.</t>
+          <t>Derrière la vitre floue, les caisses râpent le pavé. Un éclat de caisse cligne sur le verre. Nina veut une pomme du hall, maintenant, dans son sac. Elle jette tout d'un coup : la cuillère, le zip qui mord. Elle refuse de forcer, range, trouve le chapeau. Au hall, la pomme roule. Elle refuse de foncer, retrouve l'éclat. La pomme paie le début.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Les caisses du hall râpent le pavé. Même d'ici, ça sent les pommes. La bouilloire chante dans la cuisine. La vapeur fait un petit nuage. Papa essuie la table. Ça sent le thé. Une tasse fume encore. Maman plie le torchon. Le tiroir fait un petit clic. Près de la porte, la vitre est un peu floue. Tu vois le hall, Nina ? Oui. Je veux une pomme qui brille. On y va, avec le sac. En ce moment, Nina cherche le sac. Papa sort le sac bleu. Le tissu sent le coton. Prends de l'eau, le hall est long. Nina met la gourde. La gourde est froide. Elle voit une cuillère en bois. Elle la pose dans le sac. La cuillère fait un bruit dur. La cuillère reste à la cuisine. Le hall n'en a pas besoin. Nina retire la cuillère. Où est le chapeau ? Le chapeau jaune n'est pas là. Sous la chaise, peut-être. Nina se penche. Le chapeau est souple, un peu poussiéreux. Elle le secoue, tout doux. Elle le met dans le sac. Ton doudou voudra la pomme aussi. Le doudou sent le coton. Il est tout doux. Nina le met dans le sac. Tu fermes ?</t>
+          <t>Derrière la vitre floue, les caisses râpent le pavé. Même ici, ça sent la pomme du hall. Nina connaît cette cuisine, ses recoins. La bouilloire chante, petite. Un nuage de vapeur touche la vitre. Sur le verre, un éclat de caisse cligne. Il vient du hall, si près. Nina ne sait pas à quoi il servira. Papa essuie la table. La nappe sent le thé chaud. Une tasse fume près du torchon. Maman plie le torchon, sans se presser. Le tiroir fait un petit clic. Nina, tu sens la pomme ? Oui, papa. Je veux une pomme, maintenant ! On y va, avec le sac. En ce moment, Nina saisit le sac bleu. Le tissu sent le coton, un peu rêche. Prends de l'eau, le hall est long. Nina prend la gourde froide. Le bouchon est lisse sous le doigt. Je mets tout, d'un coup ! Elle pousse la gourde, trop vite. Une cuillère en bois attend près du bol. Nina la jette dans le sac. La cuillère fait un bruit dur. La cuillère reste à la cuisine. Le hall n'en a pas besoin. Nina veut fermer, sans attendre. Où est mon chapeau ? Le chapeau jaune n'est pas là. Nina bourre le sac, quand même. Le zip mord la sangle. Ça reste coincé ! Elle tire plus fort. Le zip refuse. Le sourire de Nina disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Papa se baisse à sa hauteur. Tu regardes le sac ?</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Les caisses du hall râpent le pavé. Même d'ici, ça sent les pommes. La bouilloire chante dans la cuisine. La vapeur fait un petit nuage. Papa essuie la table. Ça sent le thé. Une tasse fume encore. Maman plie le torchon. Le tiroir fait un petit clic. Près de la porte, la vitre est un peu floue. Tu vois le hall, Nina ? Oui. Je veux une pomme qui brille. On y va, avec le sac. En ce moment, Nina cherche le sac. Papa sort le sac bleu. Le tissu sent le coton. Prends de l'eau, le hall est long. Nina met la gourde. La gourde est froide. Elle voit une cuillère en bois. Elle la pose dans le sac. La cuillère fait un bruit dur. La cuillère reste à la cuisine. Le hall n'en a pas besoin. Nina retire la cuillère. Où est le chapeau ? Le chapeau jaune n'est pas là. Sous la chaise, peut-être. Nina se penche. Le chapeau est souple, un peu poussiéreux. Elle le secoue, tout doux. Elle le met dans le sac. Ton doudou voudra la pomme aussi. Le doudou sent le coton. Il est tout doux. Nina le met dans le sac. Tu fermes ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Derrière la vitre floue, les caisses râpent le pavé. Même ici, ça sent la pomme du hall. Nina connaît cette cuisine, ses recoins. La bouilloire chante, petite. Un nuage de vapeur touche la vitre. Sur le verre, un &lt;emphasis level="moderate"&gt;éclat de caisse&lt;/emphasis&gt; cligne. Il vient du hall, si près. Nina ne sait pas à quoi il servira. Papa essuie la table. La nappe sent le thé chaud. Une tasse fume près du torchon. Maman plie le torchon, sans se presser. Le tiroir fait un petit clic. Nina, tu sens la pomme ? Oui, papa. Je veux une pomme, maintenant ! On y va, avec le sac. En ce moment, Nina saisit le sac bleu. Le tissu sent le coton, un peu rêche. Prends de l'eau, le hall est long. Nina prend la gourde froide. Le bouchon est lisse sous le doigt. Je mets tout, d'un coup ! Elle pousse la gourde, trop vite. Une cuillère en bois attend près du bol. Nina la jette dans le sac. La cuillère fait un bruit dur. La cuillère reste à la cuisine. Le hall n'en a pas besoin. Nina veut fermer, sans attendre. Où est mon chapeau ? Le chapeau jaune n'est pas là. Nina bourre le sac, quand même. Le zip mord la sangle. Ça reste coincé ! Elle tire plus fort. Le zip refuse. Le sourire de Nina disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Papa se baisse à sa hauteur. Tu regardes le sac ?&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Clovis est dans l'entrée. Papa sort le &lt;emphasis&gt;sac&lt;/emphasis&gt; bleu. Papa, l'adulte, dit : on met la gourde. On met le chapeau. On met le doudou. Clovis écoute. Il met dans le sac ce que l'adulte a dit. La gourde est froide. Le chapeau est jaune. Le doudou sent le coton. Clovis ferme le sac. Parce qu'il a mis ce que papa a dit, le sac est prêt. Maman arrive. Elle dit : bravo. Ils sortent. Le sac est sur le dos de Clovis. [pause]</t>
+          <t>Derrière la vitre floue, les caisses râpent le pavé. Même ici, ça sent la pomme du hall. Nina connaît cette cuisine, ses recoins. La bouilloire chante, petite. Un nuage de vapeur touche la vitre. Sur le verre, un &lt;emphasis&gt;éclat de caisse&lt;/emphasis&gt; cligne. Il vient du hall, si près. Nina ne sait pas à quoi il servira. Papa essuie la table. La nappe sent le thé chaud. Une tasse fume près du torchon. Maman plie le torchon, sans se presser. Le tiroir fait un petit clic. Nina, tu sens la pomme ? Oui, papa. Je veux une pomme, maintenant ! On y va, avec le sac. En ce moment, Nina saisit le sac bleu. Le tissu sent le coton, un peu rêche. Prends de l'eau, le hall est long. Nina prend la gourde froide. Le bouchon est lisse sous le doigt. Je mets tout, d'un coup ! Elle pousse la gourde, trop vite. Une cuillère en bois attend près du bol. Nina la jette dans le sac. La cuillère fait un bruit dur. La cuillère reste à la cuisine. Le hall n'en a pas besoin. Nina veut fermer, sans attendre. Où est mon chapeau ? Le chapeau jaune n'est pas là. Nina bourre le sac, quand même. Le zip mord la sangle. Ça reste coincé ! Elle tire plus fort. Le zip refuse. Le sourire de Nina disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Papa se baisse à sa hauteur. Tu regardes le sac ? [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>sac</t>
+          <t>éclat de caisse</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,52 +1321,59 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=elle_veut_la_pomme_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Les caisses du hall râpent le pavé.
-narrateur|Même d'ici, ça sent les pommes.
-narrateur|La bouilloire chante dans la cuisine.
-narrateur|La vapeur fait un petit nuage.
+          <t>narrateur|Derrière la vitre floue, les caisses râpent le pavé.
+narrateur|Même ici, ça sent la pomme du hall.
+narrateur|Nina connaît cette cuisine, ses recoins.
+narrateur|La bouilloire chante, petite.
+narrateur|Un nuage de vapeur touche la vitre.
+narrateur|Sur le verre, un éclat de caisse cligne.
+narrateur|Il vient du hall, si près.
+narrateur|Nina ne sait pas à quoi il servira.
 narrateur|Papa essuie la table.
-narrateur|Ça sent le thé.
-narrateur|Une tasse fume encore.
-narrateur|Maman plie le torchon.
+narrateur|La nappe sent le thé chaud.
+narrateur|Une tasse fume près du torchon.
+narrateur|Maman plie le torchon, sans se presser.
 narrateur|Le tiroir fait un petit clic.
-narrateur|Près de la porte, la vitre est un peu floue.
-papa|Tu vois le hall, Nina ?
-enfant-f|Oui.
-enfant-f|Je veux une pomme qui brille.
+papa|Nina, tu sens la pomme ?
+enfant-f|Oui, papa.
+enfant-f|Je veux une pomme, maintenant !
 maman|On y va, avec le sac.
-narrateur|En ce moment, Nina cherche le sac.
-narrateur|Papa sort le sac bleu.
-narrateur|Le tissu sent le coton.
+narrateur|En ce moment, Nina saisit le sac bleu.
+narrateur|Le tissu sent le coton, un peu rêche.
 papa|Prends de l'eau, le hall est long.
-narrateur|Nina met la gourde.
-narrateur|La gourde est froide.
-narrateur|Elle voit une cuillère en bois.
-narrateur|Elle la pose dans le sac.
+narrateur|Nina prend la gourde froide.
+narrateur|Le bouchon est lisse sous le doigt.
+enfant-f|Je mets tout, d'un coup !
+narrateur|Elle pousse la gourde, trop vite.
+narrateur|Une cuillère en bois attend près du bol.
+narrateur|Nina la jette dans le sac.
 narrateur|La cuillère fait un bruit dur.
 papa|La cuillère reste à la cuisine.
 maman|Le hall n'en a pas besoin.
-narrateur|Nina retire la cuillère.
-enfant-f|Où est le chapeau ?
+narrateur|Nina veut fermer, sans attendre.
+enfant-f|Où est mon chapeau ?
 narrateur|Le chapeau jaune n'est pas là.
-maman|Sous la chaise, peut-être.
-narrateur|Nina se penche.
-narrateur|Le chapeau est souple, un peu poussiéreux.
-narrateur|Elle le secoue, tout doux.
-narrateur|Elle le met dans le sac.
-papa|Ton doudou voudra la pomme aussi.
-narrateur|Le doudou sent le coton.
-enfant-f|Il est tout doux.
-narrateur|Nina le met dans le sac.
-maman|Tu fermes ?</t>
+narrateur|Nina bourre le sac, quand même.
+narrateur|Le zip mord la sangle.
+enfant-f|Ça reste coincé !
+narrateur|Elle tire plus fort.
+narrateur|Le zip refuse.
+narrateur|Le sourire de Nina disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Papa se baisse à sa hauteur.
+papa|Tu regardes le sac ?</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>enfants_parc</t>
+          <t>bouilloire,caisses,vitre</t>
         </is>
       </c>
     </row>
@@ -1398,12 +1405,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Nina prépare le sac. Où met-elle les affaires ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Nina prépare le &lt;emphasis level="moderate"&gt;sac&lt;/emphasis&gt;. Où met-elle les affaires ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Papa a parlé. Que met Clovis dans le &lt;emphasis&gt;sac&lt;/emphasis&gt; ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Nina prépare le &lt;emphasis&gt;sac&lt;/emphasis&gt;. Où met-elle les affaires ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1466,7 +1473,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1477,7 +1484,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.28</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1492,11 +1499,11 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AH3" s="2" t="inlineStr">
         <is>
@@ -1507,23 +1514,23 @@
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1538,17 +1545,17 @@
         <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=les_affaires_vont_dans_le_sac; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1581,17 +1588,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Nina ferme le sac. Ça fait zzz. Le sac bleu est prêt. Le sac est prêt ? Oui, maman. Merci, Nina. Tu as laissé la cuillère ici. Le petit nuage de la bouilloire s'en va. On peut sortir, maintenant. La pomme m'attend. Oui, elle brille déjà, là-bas. Nina enfile le sac. Le sac est sur le dos de Nina. Tu as ton sac, Nina ? Oui, maman. On ouvre la porte. Papa ouvre la porte.</t>
+          <t>Nina refuse de tirer plus fort. Elle pose un genou au sol. La sangle est plate, sous le zip. Je la sors. Elle pousse le tissu, un peu. Le zip lâche, petit à petit. Il part. Sors la cuillère, d'abord. Nina retire la cuillère en bois. Elle la pose près de la tasse. Le chapeau, sous la chaise ? Nina se penche. Le chapeau est souple, un peu poussiéreux. Elle le secoue, au-dessus du sol. Le chapeau glisse dans le sac. Ton doudou voudra la pomme, lui aussi. Où est-il ? Le doudou n'est pas près des chaussures. Regarde sur la chaise, près du torchon. Nina cherche près du torchon. Le doudou sent le coton chaud. Il était caché. Elle le glisse dans le sac. La gourde reste au fond, froide. Le zip avance, sans mordre. Tu fermes, Nina ? Oui, maman. Nina appuie sur la fermeture. Ça fait un petit zzz. Le sac bleu est fermé. Merci, Nina. Le sac est prêt ? Oui, papa. Nina pose la main sur le tissu. Le tissu est un peu rêche.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Nina ferme le sac. Ça fait zzz. Le sac bleu est prêt. Le sac est prêt ? Oui, maman. Merci, Nina. Tu as laissé la cuillère ici. Le petit nuage de la bouilloire s'en va. On peut sortir, maintenant. La pomme m'attend. Oui, elle brille déjà, là-bas. Nina enfile le sac. Le sac est sur le dos de Nina. Tu as ton sac, Nina ? Oui, maman. On ouvre la porte. Papa ouvre la porte.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nina refuse de tirer plus fort. Elle pose un genou au sol. La sangle est plate, sous le zip. Je la sors. Elle pousse le tissu, un peu. Le zip lâche, petit à petit. Il part. Sors la cuillère, d'abord. Nina retire la cuillère en bois. Elle la pose près de la tasse. Le chapeau, sous la chaise ? Nina se penche. Le chapeau est souple, un peu poussiéreux. Elle le secoue, au-dessus du sol. Le chapeau glisse dans le &lt;emphasis level="moderate"&gt;sac&lt;/emphasis&gt;. Ton doudou voudra la pomme, lui aussi. Où est-il ? Le doudou n'est pas près des chaussures. Regarde sur la chaise, près du torchon. Nina cherche près du torchon. Le doudou sent le coton chaud. Il était caché. Elle le glisse dans le sac. La gourde reste au fond, froide. Le zip avance, sans mordre. Tu fermes, Nina ? Oui, maman. Nina appuie sur la fermeture. Ça fait un petit zzz. Le sac bleu est fermé. Merci, Nina. Le sac est prêt ? Oui, papa. Nina pose la main sur le tissu. Le tissu est un peu rêche.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Clovis a préparé le &lt;emphasis&gt;sac&lt;/emphasis&gt;. Il a mis ce que l'adulte a dit. Papa et maman étaient là. [pause]</t>
+          <t>Nina refuse de tirer plus fort. Elle pose un genou au sol. La sangle est plate, sous le zip. Je la sors. Elle pousse le tissu, un peu. Le zip lâche, petit à petit. Il part. Sors la cuillère, d'abord. Nina retire la cuillère en bois. Elle la pose près de la tasse. Le chapeau, sous la chaise ? Nina se penche. Le chapeau est souple, un peu poussiéreux. Elle le secoue, au-dessus du sol. Le chapeau glisse dans le &lt;emphasis&gt;sac&lt;/emphasis&gt;. Ton doudou voudra la pomme, lui aussi. Où est-il ? Le doudou n'est pas près des chaussures. Regarde sur la chaise, près du torchon. Nina cherche près du torchon. Le doudou sent le coton chaud. Il était caché. Elle le glisse dans le sac. La gourde reste au fond, froide. Le zip avance, sans mordre. Tu fermes, Nina ? Oui, maman. Nina appuie sur la fermeture. Ça fait un petit zzz. Le sac bleu est fermé. Merci, Nina. Le sac est prêt ? Oui, papa. Nina pose la main sur le tissu. Le tissu est un peu rêche. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1638,7 +1645,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1646,10 +1653,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1679,23 +1686,23 @@
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1704,10 +1711,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1720,28 +1727,51 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=concentration puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=elle_prépare_sans_foncer; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Nina ferme le sac.
-narrateur|Ça fait zzz.
-narrateur|Le sac bleu est prêt.
-maman|Le sac est prêt ?
+          <t>narrateur|Nina refuse de tirer plus fort.
+narrateur|Elle pose un genou au sol.
+narrateur|La sangle est plate, sous le zip.
+enfant-f|Je la sors.
+narrateur|Elle pousse le tissu, un peu.
+narrateur|Le zip lâche, petit à petit.
+enfant-f|Il part.
+papa|Sors la cuillère, d'abord.
+narrateur|Nina retire la cuillère en bois.
+narrateur|Elle la pose près de la tasse.
+maman|Le chapeau, sous la chaise ?
+narrateur|Nina se penche.
+narrateur|Le chapeau est souple, un peu poussiéreux.
+narrateur|Elle le secoue, au-dessus du sol.
+narrateur|Le chapeau glisse dans le sac.
+papa|Ton doudou voudra la pomme, lui aussi.
+enfant-f|Où est-il ?
+narrateur|Le doudou n'est pas près des chaussures.
+maman|Regarde sur la chaise, près du torchon.
+narrateur|Nina cherche près du torchon.
+narrateur|Le doudou sent le coton chaud.
+enfant-f|Il était caché.
+narrateur|Elle le glisse dans le sac.
+narrateur|La gourde reste au fond, froide.
+narrateur|Le zip avance, sans mordre.
+maman|Tu fermes, Nina ?
 enfant-f|Oui, maman.
+narrateur|Nina appuie sur la fermeture.
+narrateur|Ça fait un petit zzz.
+narrateur|Le sac bleu est fermé.
 papa|Merci, Nina.
-papa|Tu as laissé la cuillère ici.
-narrateur|Le petit nuage de la bouilloire s'en va.
-maman|On peut sortir, maintenant.
-enfant-f|La pomme m'attend.
-papa|Oui, elle brille déjà, là-bas.
-narrateur|Nina enfile le sac.
-narrateur|Le sac est sur le dos de Nina.
-maman|Tu as ton sac, Nina ?
-enfant-f|Oui, maman.
-papa|On ouvre la porte.
-narrateur|Papa ouvre la porte.</t>
+papa|Le sac est prêt ?
+enfant-f|Oui, papa.
+narrateur|Nina pose la main sur le tissu.
+narrateur|Le tissu est un peu rêche.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>zip,sac</t>
         </is>
       </c>
     </row>
@@ -1768,17 +1798,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Ils sortent. L'air sent les caisses et le fruit. Le hall n'est plus flou. Il est vrai, maintenant. Oui, on y va ensemble. Une pomme rouge brille sur une caisse. Nina s'accroupit. Elle touche la peau lisse. Elle est un peu froide, un peu sucrée. Elle brille, maman. Tu la choisis ? Celle-là. Nina ferme la main autour de la pomme. Le fruit reste un moment, tout rond. On la sent ensemble ? Oui. Nina approche la pomme de son nez. Ça sent le sucre et la peau. Tu l'as trouvée. Une caisse râpe encore le pavé, tout loin.</t>
+          <t>On met tes chaussures ? Nina enfile ses chaussures. Une semelle est froide. Tu as fini tes chaussures ? Oui, maman. On ouvre la porte. Papa ouvre la porte. L'air sent les caisses et le fruit. Le hall n'est plus flou. Il est vrai ! Oui, on y va ensemble. Nina enfile le sac. Le sac tape contre son dos. Ils marchent vers le hall aux caisses. Le pavé est un peu poudreux. Je la prends ! Une pomme rouge brille, trop près. Nina tend la main, trop vite. La pomme glisse, roule sous une caisse. Oh. Elle veut foncer, à quatre pattes. Nina refuse de foncer. Attends, je regarde. Sur le bois, un éclat de caisse cligne. C'est celui de la vitre. Comme à la cuisine ! Tu le vois, toi ? Oui, sur cette caisse. Nina s'accroupit, lente. Elle écoute le hall, un instant. Une autre caisse râpe, plus loin. La pomme attend sous le bois. Nina glisse la main, lente. Ses doigts trouvent la peau lisse.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Ils sortent. L'air sent les caisses et le fruit. Le hall n'est plus flou. Il est vrai, maintenant. Oui, on y va ensemble. Une pomme rouge brille sur une caisse. Nina s'accroupit. Elle touche la peau lisse. Elle est un peu froide, un peu sucrée. Elle brille, maman. Tu la choisis ? Celle-là. Nina ferme la main autour de la pomme. Le fruit reste un moment, tout rond. On la sent ensemble ? Oui. Nina approche la pomme de son nez. Ça sent le sucre et la peau. Tu l'as trouvée. Une caisse râpe encore le pavé, tout loin.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;On met tes chaussures ? Nina enfile ses chaussures. Une semelle est froide. Tu as fini tes chaussures ? Oui, maman. On ouvre la porte. Papa ouvre la porte. L'air sent les caisses et le fruit. Le hall n'est plus flou. Il est vrai ! Oui, on y va ensemble. Nina enfile le sac. Le sac tape contre son dos. Ils marchent vers le hall aux caisses. Le pavé est un peu poudreux. Je la prends ! Une pomme rouge brille, trop près. Nina tend la main, trop vite. La pomme glisse, roule sous une caisse. Oh. Elle veut foncer, à quatre pattes. Nina refuse de foncer. Attends, je regarde. Sur le bois, un &lt;emphasis level="moderate"&gt;éclat de caisse&lt;/emphasis&gt; cligne. C'est celui de la vitre. Comme à la cuisine ! Tu le vois, toi ? Oui, sur cette caisse. Nina s'accroupit, lente. Elle écoute le hall, un instant. Une autre caisse râpe, plus loin. La pomme attend sous le bois. Nina glisse la main, lente. Ses doigts trouvent la peau lisse.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Clovis enfile le &lt;emphasis&gt;sac&lt;/emphasis&gt;. Papa ouvre la porte. [pause]</t>
+          <t>&lt;low-pitch&gt;On met tes chaussures ? Nina enfile ses chaussures. Une semelle est froide. Tu as fini tes chaussures ? Oui, maman. On ouvre la porte. Papa ouvre la porte. L'air sent les caisses et le fruit. Le hall n'est plus flou. Il est vrai ! Oui, on y va ensemble. Nina enfile le sac. Le sac tape contre son dos. Ils marchent vers le hall aux caisses. Le pavé est un peu poudreux. Je la prends ! Une pomme rouge brille, trop près. Nina tend la main, trop vite. La pomme glisse, roule sous une caisse. Oh. Elle veut foncer, à quatre pattes. Nina refuse de foncer. Attends, je regarde. Sur le bois, un &lt;emphasis&gt;éclat de caisse&lt;/emphasis&gt; cligne. C'est celui de la vitre. Comme à la cuisine ! Tu le vois, toi ? Oui, sur cette caisse. Nina s'accroupit, lente. Elle écoute le hall, un instant. Une autre caisse râpe, plus loin. La pomme attend sous le bois. Nina glisse la main, lente. Ses doigts trouvent la peau lisse.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1825,7 +1855,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1833,22 +1863,26 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.18</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AE5" s="2" t="inlineStr"/>
+          <t>-2st</t>
+        </is>
+      </c>
+      <c r="AE5" s="2" t="inlineStr">
+        <is>
+          <t>low-pitch</t>
+        </is>
+      </c>
       <c r="AF5" s="2" t="inlineStr">
         <is>
           <t>medium</t>
@@ -1859,30 +1893,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>sac</t>
+          <t>éclat de caisse</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>520</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>300</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>tense</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1891,43 +1925,66 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
       </c>
       <c r="AT5" s="2" t="n">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=obstacle; intention=alerter_sans_effrayer; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=elle_refuse_de_foncer_retrouve_l_eclat; tempo=resserré; sourire=aucun; respiration=retenue</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Ils sortent.
+          <t>papa|On met tes chaussures ?
+narrateur|Nina enfile ses chaussures.
+narrateur|Une semelle est froide.
+maman|Tu as fini tes chaussures ?
+enfant-f|Oui, maman.
+papa|On ouvre la porte.
+narrateur|Papa ouvre la porte.
 narrateur|L'air sent les caisses et le fruit.
 narrateur|Le hall n'est plus flou.
-enfant-f|Il est vrai, maintenant.
+enfant-f|Il est vrai !
 papa|Oui, on y va ensemble.
-narrateur|Une pomme rouge brille sur une caisse.
-narrateur|Nina s'accroupit.
-narrateur|Elle touche la peau lisse.
-narrateur|Elle est un peu froide, un peu sucrée.
-enfant-f|Elle brille, maman.
-maman|Tu la choisis ?
-enfant-f|Celle-là.
-narrateur|Nina ferme la main autour de la pomme.
-narrateur|Le fruit reste un moment, tout rond.
-papa|On la sent ensemble ?
-enfant-f|Oui.
-narrateur|Nina approche la pomme de son nez.
-narrateur|Ça sent le sucre et la peau.
-maman|Tu l'as trouvée.
-narrateur|Une caisse râpe encore le pavé, tout loin.</t>
+narrateur|Nina enfile le sac.
+narrateur|Le sac tape contre son dos.
+narrateur|Ils marchent vers le hall aux caisses.
+narrateur|Le pavé est un peu poudreux.
+enfant-f|Je la prends !
+narrateur|Une pomme rouge brille, trop près.
+narrateur|Nina tend la main, trop vite.
+narrateur|La pomme glisse, roule sous une caisse.
+enfant-f|Oh.
+narrateur|Elle veut foncer, à quatre pattes.
+narrateur|Nina refuse de foncer.
+enfant-f|Attends, je regarde.
+narrateur|Sur le bois, un éclat de caisse cligne.
+narrateur|C'est celui de la vitre.
+enfant-f|Comme à la cuisine !
+maman|Tu le vois, toi ?
+enfant-f|Oui, sur cette caisse.
+narrateur|Nina s'accroupit, lente.
+narrateur|Elle écoute le hall, un instant.
+narrateur|Une autre caisse râpe, plus loin.
+narrateur|La pomme attend sous le bois.
+narrateur|Nina glisse la main, lente.
+narrateur|Ses doigts trouvent la peau lisse.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>hall,caisses,pas</t>
         </is>
       </c>
     </row>
@@ -1954,17 +2011,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Nina ouvre encore la main. La pomme rouge brille dans sa paume. Elle est à moi. Oui, tu es arrivée au hall. Le sac bleu tape le dos de Nina. Le thé de la cuisine est loin, maintenant. Merci pour le sac, Nina. La peau lisse reste froide contre sa main.</t>
+          <t>Nina ferme la main autour de la pomme. Le fruit reste rond, un peu froid. Elle brille, maman. Tu la choisis ? Celle-là. On la sent ensemble ? Oui. Nina approche la pomme de son nez. Ça sent le sucre et la peau. Sur le bois, l'éclat de caisse reste. Comme sur la vitre, papa. Tu le portes, toi ? Oui, dans mon sac. Nina ouvre le sac, un peu. Elle glisse la pomme contre le doudou. Le sac repose contre sa hanche. On la sent, papa. Tu la sens sur tes joues ? Oui, elle est froide. L'éclat de caisse laisse une trace claire, sur la peau.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Nina ouvre encore la main. La pomme rouge brille dans sa paume. Elle est à moi. Oui, tu es arrivée au hall. Le sac bleu tape le dos de Nina. Le thé de la cuisine est loin, maintenant. Merci pour le sac, Nina. La peau lisse reste froide contre sa main.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Nina ferme la main autour de la pomme. Le fruit reste rond, un peu froid. Elle brille, maman. Tu la choisis ? Celle-là. On la sent ensemble ? Oui. Nina approche la pomme de son nez. Ça sent le sucre et la peau. Sur le bois, l'&lt;emphasis level="moderate"&gt;éclat de caisse&lt;/emphasis&gt; reste. Comme sur la vitre, papa. Tu le portes, toi ? Oui, dans mon sac. Nina ouvre le sac, un peu. Elle glisse la pomme contre le doudou. Le sac repose contre sa hanche. On la sent, papa. Tu la sens sur tes joues ? Oui, elle est froide. L'éclat de caisse laisse une trace claire, sur la peau.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Nina ferme la main autour de la pomme. Le fruit reste rond, un peu froid. Elle brille, maman. Tu la choisis ? Celle-là. On la sent ensemble ? Oui. Nina approche la pomme de son nez. Ça sent le sucre et la peau. Sur le bois, l'&lt;emphasis&gt;éclat de caisse&lt;/emphasis&gt; reste. Comme sur la vitre, papa. Tu le portes, toi ? Oui, dans mon sac. Nina ouvre le sac, un peu. Elle glisse la pomme contre le doudou. Le sac repose contre sa hanche. On la sent, papa. Tu la sens sur tes joues ? Oui, elle est froide. L'éclat de caisse laisse une trace claire, sur la peau.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2011,18 +2068,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.22</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2031,12 +2088,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2045,17 +2102,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de caisse</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2064,11 +2125,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2077,31 +2138,52 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_de_la_vitre_est_sur_la_caisse; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|Nina ouvre encore la main.
-narrateur|La pomme rouge brille dans sa paume.
-enfant-f|Elle est à moi.
-papa|Oui, tu es arrivée au hall.
-narrateur|Le sac bleu tape le dos de Nina.
-narrateur|Le thé de la cuisine est loin, maintenant.
-maman|Merci pour le sac, Nina.
-narrateur|La peau lisse reste froide contre sa main.</t>
+          <t>narrateur|Nina ferme la main autour de la pomme.
+narrateur|Le fruit reste rond, un peu froid.
+enfant-f|Elle brille, maman.
+maman|Tu la choisis ?
+enfant-f|Celle-là.
+papa|On la sent ensemble ?
+enfant-f|Oui.
+narrateur|Nina approche la pomme de son nez.
+narrateur|Ça sent le sucre et la peau.
+narrateur|Sur le bois, l'éclat de caisse reste.
+enfant-f|Comme sur la vitre, papa.
+papa|Tu le portes, toi ?
+enfant-f|Oui, dans mon sac.
+narrateur|Nina ouvre le sac, un peu.
+narrateur|Elle glisse la pomme contre le doudou.
+narrateur|Le sac repose contre sa hanche.
+enfant-f|On la sent, papa.
+maman|Tu la sens sur tes joues ?
+enfant-f|Oui, elle est froide.
+narrateur|L'éclat de caisse laisse une trace claire, sur la peau.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>pomme,caisse</t>
         </is>
       </c>
     </row>
@@ -2122,7 +2204,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2214,6 +2296,13 @@
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>